<commit_message>
Envoie Commit et tâche fait.
</commit_message>
<xml_diff>
--- a/Documents/Taches.xlsx
+++ b/Documents/Taches.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chacy\My Shit\Projet1_Jeux_Video\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\travail\Projet1_Jeux_Video\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57066389-FF95-47E9-9DF2-5068CA0985FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF794A21-7105-4B53-8F34-AC39B9AA0D46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3BCE4F66-BD57-4DA1-9203-FCE236D7FCD6}"/>
   </bookViews>
@@ -924,7 +924,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>51</v>
@@ -939,7 +939,7 @@
         <v>47</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D3" s="15" t="s">
         <v>51</v>
@@ -1164,7 +1164,7 @@
         <v>36</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D18" s="16" t="s">
         <v>51</v>
@@ -1206,7 +1206,7 @@
         <v>42</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D21" s="8" t="s">
         <v>51</v>

</xml_diff>